<commit_message>
Add drop robot auto-generation for AB/RQM/Aux_Cycle/Mem_Cycle sections
AB starts at _16, Mem_Cycle includes JOB number. Updated Robot_Drop reference.
Synced Claude memory files.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Robot_Drop.xlsx
+++ b/Robot_Drop.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Claude Workspace\Station DB AWL Generation\Source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB75D94A-3106-45BD-9150-686EA33A51C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289EFF05-B3B4-4D87-B029-C95A71F76633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="12645" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AB" sheetId="1" r:id="rId1"/>
@@ -29,10 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="86">
-  <si>
-    <t>_06</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="75">
   <si>
     <t>BOOL</t>
   </si>
@@ -40,45 +37,12 @@
     <t>FALSE</t>
   </si>
   <si>
-    <t>_07</t>
-  </si>
-  <si>
-    <t>_08</t>
-  </si>
-  <si>
-    <t>_09</t>
-  </si>
-  <si>
     <t>RESERVE</t>
   </si>
   <si>
-    <t>_10</t>
-  </si>
-  <si>
-    <t>_11</t>
-  </si>
-  <si>
-    <t>_12</t>
-  </si>
-  <si>
-    <t>_13</t>
-  </si>
-  <si>
-    <t>_14</t>
-  </si>
-  <si>
-    <t>_15</t>
-  </si>
-  <si>
-    <t>_04</t>
-  </si>
-  <si>
     <t>CHECK STATION AND MODEL BEFORE CONSENT TO 35R01</t>
   </si>
   <si>
-    <t>_05</t>
-  </si>
-  <si>
     <t>CONSENT TO DROP PART 035R01 (JOB3)</t>
   </si>
   <si>
@@ -283,10 +247,13 @@
     <t>Clamps ready to tooling 040R03</t>
   </si>
   <si>
-    <t>MEMORY END JOB 035R01 Part dropped on 040T01</t>
-  </si>
-  <si>
-    <t>MEMORY END JOB 040R03 Part dropped on 040T01</t>
+    <t>_21</t>
+  </si>
+  <si>
+    <t>MEMORY END JOB 035R01  JOB3 Part dropped on 040T01</t>
+  </si>
+  <si>
+    <t>MEMORY END JOB 040R03 JOB2 Part dropped on 040T01</t>
   </si>
 </sst>
 </file>
@@ -618,240 +585,240 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
         <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
-        <v>2</v>
-      </c>
-      <c r="D7" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
         <v>2</v>
-      </c>
-      <c r="D8" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
         <v>2</v>
-      </c>
-      <c r="D9" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
         <v>2</v>
-      </c>
-      <c r="D10" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C17" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -870,170 +837,170 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
         <v>2</v>
-      </c>
-      <c r="D6" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
         <v>2</v>
-      </c>
-      <c r="D12" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1065,198 +1032,198 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="B8" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="B9" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="B11" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="B12" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="B15" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C17" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="B18" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1270,35 +1237,35 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="45.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>